<commit_message>
Auto-registro SGC: Folio INC-2026-0002
</commit_message>
<xml_diff>
--- a/BD_Atados_Incoming.xlsx
+++ b/BD_Atados_Incoming.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W49"/>
+  <dimension ref="A1:W97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5088,6 +5088,4566 @@
         </is>
       </c>
       <c r="W49" t="inlineStr">
+        <is>
+          <t>Material con daños en el acabado (oxido)</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>45</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A01</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>ACEROMEX-49-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E50" t="n">
+        <v>1</v>
+      </c>
+      <c r="F50" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G50" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I50" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J50" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K50" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L50" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M50" t="n">
+        <v>48</v>
+      </c>
+      <c r="N50" t="n">
+        <v>120</v>
+      </c>
+      <c r="O50" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P50" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q50" t="n">
+        <v>0</v>
+      </c>
+      <c r="R50" t="n">
+        <v>60</v>
+      </c>
+      <c r="S50" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T50" t="inlineStr">
+        <is>
+          <t>Rayas/Manchas, Marcas de Rodillos</t>
+        </is>
+      </c>
+      <c r="U50" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V50" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="W50" t="inlineStr">
+        <is>
+          <t>Material con daños en el acabado (oxido)</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>45</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A01</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>ACEROMEX-49-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E51" t="n">
+        <v>2</v>
+      </c>
+      <c r="F51" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I51" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J51" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K51" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L51" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M51" t="n">
+        <v>48</v>
+      </c>
+      <c r="N51" t="n">
+        <v>120</v>
+      </c>
+      <c r="O51" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P51" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q51" t="n">
+        <v>0</v>
+      </c>
+      <c r="R51" t="n">
+        <v>60</v>
+      </c>
+      <c r="S51" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T51" t="inlineStr">
+        <is>
+          <t>Rayas/Manchas, Marcas de Rodillos</t>
+        </is>
+      </c>
+      <c r="U51" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V51" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="W51" t="inlineStr">
+        <is>
+          <t>Material con daños en el acabado (oxido)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>45</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A01</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>ACEROMEX-49-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E52" t="n">
+        <v>3</v>
+      </c>
+      <c r="F52" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I52" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J52" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K52" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L52" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M52" t="n">
+        <v>48</v>
+      </c>
+      <c r="N52" t="n">
+        <v>120</v>
+      </c>
+      <c r="O52" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P52" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q52" t="n">
+        <v>0</v>
+      </c>
+      <c r="R52" t="n">
+        <v>60</v>
+      </c>
+      <c r="S52" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T52" t="inlineStr">
+        <is>
+          <t>Rayas/Manchas, Marcas de Rodillos</t>
+        </is>
+      </c>
+      <c r="U52" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V52" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="W52" t="inlineStr">
+        <is>
+          <t>Material con daños en el acabado (oxido)</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>45</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A01</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>ACEROMEX-49-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E53" t="n">
+        <v>4</v>
+      </c>
+      <c r="F53" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I53" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J53" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K53" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L53" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M53" t="n">
+        <v>48</v>
+      </c>
+      <c r="N53" t="n">
+        <v>120</v>
+      </c>
+      <c r="O53" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P53" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q53" t="n">
+        <v>0</v>
+      </c>
+      <c r="R53" t="n">
+        <v>60</v>
+      </c>
+      <c r="S53" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T53" t="inlineStr">
+        <is>
+          <t>Rayas/Manchas, Marcas de Rodillos</t>
+        </is>
+      </c>
+      <c r="U53" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V53" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="W53" t="inlineStr">
+        <is>
+          <t>Material con daños en el acabado (oxido)</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>45</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A02</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>ACEROMEX-50-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E54" t="n">
+        <v>1</v>
+      </c>
+      <c r="F54" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G54" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I54" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J54" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K54" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L54" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M54" t="n">
+        <v>48</v>
+      </c>
+      <c r="N54" t="n">
+        <v>120</v>
+      </c>
+      <c r="O54" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P54" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q54" t="n">
+        <v>0</v>
+      </c>
+      <c r="R54" t="n">
+        <v>60</v>
+      </c>
+      <c r="S54" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T54" t="inlineStr">
+        <is>
+          <t>Rayas/Manchas, Marcas de Rodillos</t>
+        </is>
+      </c>
+      <c r="U54" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V54" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="W54" t="inlineStr">
+        <is>
+          <t>Material con daños en el acabado (oxido)</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>45</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A02</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>ACEROMEX-50-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E55" t="n">
+        <v>2</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J55" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K55" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L55" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M55" t="n">
+        <v>48</v>
+      </c>
+      <c r="N55" t="n">
+        <v>120</v>
+      </c>
+      <c r="O55" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P55" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q55" t="n">
+        <v>0</v>
+      </c>
+      <c r="R55" t="n">
+        <v>60</v>
+      </c>
+      <c r="S55" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T55" t="inlineStr">
+        <is>
+          <t>Rayas/Manchas, Marcas de Rodillos</t>
+        </is>
+      </c>
+      <c r="U55" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V55" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="W55" t="inlineStr">
+        <is>
+          <t>Material con daños en el acabado (oxido)</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>45</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A02</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>ACEROMEX-50-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E56" t="n">
+        <v>3</v>
+      </c>
+      <c r="F56" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G56" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J56" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K56" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L56" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M56" t="n">
+        <v>48</v>
+      </c>
+      <c r="N56" t="n">
+        <v>120</v>
+      </c>
+      <c r="O56" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P56" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q56" t="n">
+        <v>0</v>
+      </c>
+      <c r="R56" t="n">
+        <v>60</v>
+      </c>
+      <c r="S56" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T56" t="inlineStr">
+        <is>
+          <t>Rayas/Manchas, Marcas de Rodillos</t>
+        </is>
+      </c>
+      <c r="U56" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V56" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="W56" t="inlineStr">
+        <is>
+          <t>Material con daños en el acabado (oxido)</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>45</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A02</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>ACEROMEX-50-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E57" t="n">
+        <v>4</v>
+      </c>
+      <c r="F57" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G57" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J57" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K57" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L57" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M57" t="n">
+        <v>48</v>
+      </c>
+      <c r="N57" t="n">
+        <v>120</v>
+      </c>
+      <c r="O57" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P57" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q57" t="n">
+        <v>0</v>
+      </c>
+      <c r="R57" t="n">
+        <v>60</v>
+      </c>
+      <c r="S57" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T57" t="inlineStr">
+        <is>
+          <t>Rayas/Manchas, Marcas de Rodillos</t>
+        </is>
+      </c>
+      <c r="U57" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V57" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="W57" t="inlineStr">
+        <is>
+          <t>Material con daños en el acabado (oxido)</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>45</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A03</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>ACEROMEX-51-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E58" t="n">
+        <v>1</v>
+      </c>
+      <c r="F58" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G58" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J58" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K58" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L58" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M58" t="n">
+        <v>48</v>
+      </c>
+      <c r="N58" t="n">
+        <v>120</v>
+      </c>
+      <c r="O58" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P58" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q58" t="n">
+        <v>0</v>
+      </c>
+      <c r="R58" t="n">
+        <v>60</v>
+      </c>
+      <c r="S58" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T58" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U58" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V58" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W58" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>45</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A03</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>ACEROMEX-51-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E59" t="n">
+        <v>2</v>
+      </c>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G59" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J59" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K59" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L59" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M59" t="n">
+        <v>48</v>
+      </c>
+      <c r="N59" t="n">
+        <v>120</v>
+      </c>
+      <c r="O59" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P59" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q59" t="n">
+        <v>0</v>
+      </c>
+      <c r="R59" t="n">
+        <v>60</v>
+      </c>
+      <c r="S59" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T59" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U59" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V59" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W59" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>45</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A03</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>ACEROMEX-51-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E60" t="n">
+        <v>3</v>
+      </c>
+      <c r="F60" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J60" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K60" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L60" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M60" t="n">
+        <v>48</v>
+      </c>
+      <c r="N60" t="n">
+        <v>120</v>
+      </c>
+      <c r="O60" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P60" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q60" t="n">
+        <v>0</v>
+      </c>
+      <c r="R60" t="n">
+        <v>60</v>
+      </c>
+      <c r="S60" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T60" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U60" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V60" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W60" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>45</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A03</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>ACEROMEX-51-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E61" t="n">
+        <v>4</v>
+      </c>
+      <c r="F61" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G61" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J61" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K61" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L61" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M61" t="n">
+        <v>48</v>
+      </c>
+      <c r="N61" t="n">
+        <v>120</v>
+      </c>
+      <c r="O61" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P61" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q61" t="n">
+        <v>0</v>
+      </c>
+      <c r="R61" t="n">
+        <v>60</v>
+      </c>
+      <c r="S61" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T61" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U61" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V61" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W61" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>45</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A04</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>ACEROMEX-52-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E62" t="n">
+        <v>1</v>
+      </c>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J62" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K62" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L62" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M62" t="n">
+        <v>48</v>
+      </c>
+      <c r="N62" t="n">
+        <v>120</v>
+      </c>
+      <c r="O62" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P62" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q62" t="n">
+        <v>0</v>
+      </c>
+      <c r="R62" t="n">
+        <v>60</v>
+      </c>
+      <c r="S62" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T62" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U62" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V62" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W62" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>45</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A04</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>ACEROMEX-52-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E63" t="n">
+        <v>2</v>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J63" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K63" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L63" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M63" t="n">
+        <v>48</v>
+      </c>
+      <c r="N63" t="n">
+        <v>120</v>
+      </c>
+      <c r="O63" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P63" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q63" t="n">
+        <v>0</v>
+      </c>
+      <c r="R63" t="n">
+        <v>60</v>
+      </c>
+      <c r="S63" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T63" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U63" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V63" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W63" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>45</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A04</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>ACEROMEX-52-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E64" t="n">
+        <v>3</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J64" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K64" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L64" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M64" t="n">
+        <v>48</v>
+      </c>
+      <c r="N64" t="n">
+        <v>120</v>
+      </c>
+      <c r="O64" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P64" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q64" t="n">
+        <v>0</v>
+      </c>
+      <c r="R64" t="n">
+        <v>60</v>
+      </c>
+      <c r="S64" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T64" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U64" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V64" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W64" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>45</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A04</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>ACEROMEX-52-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E65" t="n">
+        <v>4</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J65" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K65" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L65" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M65" t="n">
+        <v>48</v>
+      </c>
+      <c r="N65" t="n">
+        <v>120</v>
+      </c>
+      <c r="O65" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P65" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q65" t="n">
+        <v>0</v>
+      </c>
+      <c r="R65" t="n">
+        <v>60</v>
+      </c>
+      <c r="S65" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T65" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U65" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V65" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W65" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>45</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A05</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>ACEROMEX-53-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E66" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J66" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K66" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L66" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M66" t="n">
+        <v>48</v>
+      </c>
+      <c r="N66" t="n">
+        <v>120</v>
+      </c>
+      <c r="O66" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P66" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q66" t="n">
+        <v>0</v>
+      </c>
+      <c r="R66" t="n">
+        <v>60</v>
+      </c>
+      <c r="S66" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T66" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U66" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V66" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W66" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>45</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A05</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>ACEROMEX-53-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E67" t="n">
+        <v>2</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J67" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K67" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L67" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M67" t="n">
+        <v>48</v>
+      </c>
+      <c r="N67" t="n">
+        <v>120</v>
+      </c>
+      <c r="O67" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P67" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q67" t="n">
+        <v>0</v>
+      </c>
+      <c r="R67" t="n">
+        <v>60</v>
+      </c>
+      <c r="S67" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T67" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U67" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V67" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W67" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>45</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A05</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>ACEROMEX-53-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E68" t="n">
+        <v>3</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J68" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K68" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L68" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M68" t="n">
+        <v>48</v>
+      </c>
+      <c r="N68" t="n">
+        <v>120</v>
+      </c>
+      <c r="O68" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P68" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q68" t="n">
+        <v>0</v>
+      </c>
+      <c r="R68" t="n">
+        <v>60</v>
+      </c>
+      <c r="S68" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T68" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U68" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V68" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W68" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>45</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A05</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>ACEROMEX-53-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E69" t="n">
+        <v>4</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J69" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K69" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L69" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M69" t="n">
+        <v>48</v>
+      </c>
+      <c r="N69" t="n">
+        <v>120</v>
+      </c>
+      <c r="O69" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P69" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q69" t="n">
+        <v>0</v>
+      </c>
+      <c r="R69" t="n">
+        <v>60</v>
+      </c>
+      <c r="S69" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T69" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U69" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V69" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W69" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>45</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A06</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>ACEROMEX-54-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E70" t="n">
+        <v>1</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J70" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K70" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L70" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M70" t="n">
+        <v>48</v>
+      </c>
+      <c r="N70" t="n">
+        <v>120</v>
+      </c>
+      <c r="O70" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P70" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q70" t="n">
+        <v>0</v>
+      </c>
+      <c r="R70" t="n">
+        <v>60</v>
+      </c>
+      <c r="S70" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T70" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U70" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V70" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W70" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>45</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A06</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>ACEROMEX-54-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E71" t="n">
+        <v>2</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J71" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K71" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L71" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M71" t="n">
+        <v>48</v>
+      </c>
+      <c r="N71" t="n">
+        <v>120</v>
+      </c>
+      <c r="O71" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P71" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q71" t="n">
+        <v>0</v>
+      </c>
+      <c r="R71" t="n">
+        <v>60</v>
+      </c>
+      <c r="S71" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T71" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U71" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V71" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W71" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>45</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A06</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>ACEROMEX-54-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E72" t="n">
+        <v>3</v>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J72" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K72" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L72" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M72" t="n">
+        <v>48</v>
+      </c>
+      <c r="N72" t="n">
+        <v>120</v>
+      </c>
+      <c r="O72" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P72" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q72" t="n">
+        <v>0</v>
+      </c>
+      <c r="R72" t="n">
+        <v>60</v>
+      </c>
+      <c r="S72" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T72" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U72" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V72" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W72" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>45</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A06</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>ACEROMEX-54-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E73" t="n">
+        <v>4</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J73" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K73" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L73" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M73" t="n">
+        <v>48</v>
+      </c>
+      <c r="N73" t="n">
+        <v>120</v>
+      </c>
+      <c r="O73" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P73" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q73" t="n">
+        <v>0</v>
+      </c>
+      <c r="R73" t="n">
+        <v>60</v>
+      </c>
+      <c r="S73" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T73" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U73" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V73" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W73" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>45</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A07</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>ACEROMEX-57-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E74" t="n">
+        <v>1</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J74" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K74" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L74" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M74" t="n">
+        <v>48</v>
+      </c>
+      <c r="N74" t="n">
+        <v>120</v>
+      </c>
+      <c r="O74" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P74" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q74" t="n">
+        <v>0</v>
+      </c>
+      <c r="R74" t="n">
+        <v>60</v>
+      </c>
+      <c r="S74" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T74" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U74" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V74" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W74" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>45</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A07</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>ACEROMEX-57-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E75" t="n">
+        <v>2</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J75" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K75" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L75" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M75" t="n">
+        <v>48</v>
+      </c>
+      <c r="N75" t="n">
+        <v>120</v>
+      </c>
+      <c r="O75" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P75" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q75" t="n">
+        <v>0</v>
+      </c>
+      <c r="R75" t="n">
+        <v>60</v>
+      </c>
+      <c r="S75" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T75" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U75" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V75" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W75" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>45</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A07</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>ACEROMEX-57-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E76" t="n">
+        <v>3</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J76" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K76" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L76" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M76" t="n">
+        <v>48</v>
+      </c>
+      <c r="N76" t="n">
+        <v>120</v>
+      </c>
+      <c r="O76" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P76" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q76" t="n">
+        <v>0</v>
+      </c>
+      <c r="R76" t="n">
+        <v>60</v>
+      </c>
+      <c r="S76" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T76" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U76" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V76" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W76" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>45</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A07</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>ACEROMEX-57-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E77" t="n">
+        <v>4</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G77" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J77" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K77" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L77" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M77" t="n">
+        <v>48</v>
+      </c>
+      <c r="N77" t="n">
+        <v>120</v>
+      </c>
+      <c r="O77" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P77" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q77" t="n">
+        <v>0</v>
+      </c>
+      <c r="R77" t="n">
+        <v>60</v>
+      </c>
+      <c r="S77" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T77" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U77" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V77" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W77" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>8</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A08</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>ACEROMEX-58-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E78" t="n">
+        <v>1</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G78" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J78" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K78" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L78" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M78" t="n">
+        <v>48</v>
+      </c>
+      <c r="N78" t="n">
+        <v>120</v>
+      </c>
+      <c r="O78" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P78" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q78" t="n">
+        <v>0</v>
+      </c>
+      <c r="R78" t="n">
+        <v>60</v>
+      </c>
+      <c r="S78" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T78" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U78" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V78" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W78" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>8</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A08</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>ACEROMEX-58-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E79" t="n">
+        <v>2</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G79" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J79" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K79" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L79" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M79" t="n">
+        <v>48</v>
+      </c>
+      <c r="N79" t="n">
+        <v>120</v>
+      </c>
+      <c r="O79" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P79" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q79" t="n">
+        <v>0</v>
+      </c>
+      <c r="R79" t="n">
+        <v>60</v>
+      </c>
+      <c r="S79" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T79" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U79" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V79" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W79" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>8</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A08</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>ACEROMEX-58-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E80" t="n">
+        <v>3</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J80" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K80" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L80" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M80" t="n">
+        <v>48</v>
+      </c>
+      <c r="N80" t="n">
+        <v>120</v>
+      </c>
+      <c r="O80" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P80" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q80" t="n">
+        <v>0</v>
+      </c>
+      <c r="R80" t="n">
+        <v>60</v>
+      </c>
+      <c r="S80" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T80" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U80" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V80" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W80" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>8</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A08</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>ACEROMEX-58-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E81" t="n">
+        <v>4</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G81" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J81" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K81" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L81" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M81" t="n">
+        <v>48</v>
+      </c>
+      <c r="N81" t="n">
+        <v>120</v>
+      </c>
+      <c r="O81" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P81" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q81" t="n">
+        <v>0</v>
+      </c>
+      <c r="R81" t="n">
+        <v>60</v>
+      </c>
+      <c r="S81" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T81" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U81" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V81" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W81" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>45</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A09</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>ACEROMEX-59-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E82" t="n">
+        <v>1</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G82" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J82" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K82" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L82" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M82" t="n">
+        <v>48</v>
+      </c>
+      <c r="N82" t="n">
+        <v>120</v>
+      </c>
+      <c r="O82" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P82" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q82" t="n">
+        <v>0</v>
+      </c>
+      <c r="R82" t="n">
+        <v>60</v>
+      </c>
+      <c r="S82" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T82" t="inlineStr">
+        <is>
+          <t>Rayas/Manchas, Marcas de Rodillos</t>
+        </is>
+      </c>
+      <c r="U82" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V82" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="W82" t="inlineStr">
+        <is>
+          <t>Material con daños en el acabado (rayones profundos )</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>45</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A09</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>ACEROMEX-59-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E83" t="n">
+        <v>2</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G83" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J83" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K83" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L83" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M83" t="n">
+        <v>48</v>
+      </c>
+      <c r="N83" t="n">
+        <v>120</v>
+      </c>
+      <c r="O83" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P83" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q83" t="n">
+        <v>0</v>
+      </c>
+      <c r="R83" t="n">
+        <v>60</v>
+      </c>
+      <c r="S83" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T83" t="inlineStr">
+        <is>
+          <t>Rayas/Manchas, Marcas de Rodillos</t>
+        </is>
+      </c>
+      <c r="U83" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V83" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="W83" t="inlineStr">
+        <is>
+          <t>Material con daños en el acabado (rayones profundos )</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>45</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A09</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>ACEROMEX-59-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E84" t="n">
+        <v>3</v>
+      </c>
+      <c r="F84" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G84" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J84" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K84" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L84" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M84" t="n">
+        <v>48</v>
+      </c>
+      <c r="N84" t="n">
+        <v>120</v>
+      </c>
+      <c r="O84" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P84" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q84" t="n">
+        <v>0</v>
+      </c>
+      <c r="R84" t="n">
+        <v>60</v>
+      </c>
+      <c r="S84" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T84" t="inlineStr">
+        <is>
+          <t>Rayas/Manchas, Marcas de Rodillos</t>
+        </is>
+      </c>
+      <c r="U84" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V84" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="W84" t="inlineStr">
+        <is>
+          <t>Material con daños en el acabado (rayones profundos )</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>45</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A09</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>ACEROMEX-59-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E85" t="n">
+        <v>4</v>
+      </c>
+      <c r="F85" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G85" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J85" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K85" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L85" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M85" t="n">
+        <v>48</v>
+      </c>
+      <c r="N85" t="n">
+        <v>120</v>
+      </c>
+      <c r="O85" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P85" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q85" t="n">
+        <v>0</v>
+      </c>
+      <c r="R85" t="n">
+        <v>60</v>
+      </c>
+      <c r="S85" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T85" t="inlineStr">
+        <is>
+          <t>Rayas/Manchas, Marcas de Rodillos</t>
+        </is>
+      </c>
+      <c r="U85" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V85" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="W85" t="inlineStr">
+        <is>
+          <t>Material con daños en el acabado (rayones profundos )</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>45</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A10</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D86" t="inlineStr">
+        <is>
+          <t>ACEROMEX-64-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E86" t="n">
+        <v>1</v>
+      </c>
+      <c r="F86" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G86" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J86" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K86" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L86" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M86" t="n">
+        <v>48</v>
+      </c>
+      <c r="N86" t="n">
+        <v>120</v>
+      </c>
+      <c r="O86" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P86" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q86" t="n">
+        <v>0</v>
+      </c>
+      <c r="R86" t="n">
+        <v>60</v>
+      </c>
+      <c r="S86" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T86" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U86" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V86" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W86" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="n">
+        <v>45</v>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A10</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>ACEROMEX-64-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E87" t="n">
+        <v>2</v>
+      </c>
+      <c r="F87" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G87" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J87" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K87" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L87" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M87" t="n">
+        <v>48</v>
+      </c>
+      <c r="N87" t="n">
+        <v>120</v>
+      </c>
+      <c r="O87" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P87" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q87" t="n">
+        <v>0</v>
+      </c>
+      <c r="R87" t="n">
+        <v>60</v>
+      </c>
+      <c r="S87" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T87" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U87" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V87" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W87" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="n">
+        <v>45</v>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A10</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>ACEROMEX-64-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E88" t="n">
+        <v>3</v>
+      </c>
+      <c r="F88" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G88" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J88" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K88" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L88" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M88" t="n">
+        <v>48</v>
+      </c>
+      <c r="N88" t="n">
+        <v>120</v>
+      </c>
+      <c r="O88" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P88" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q88" t="n">
+        <v>0</v>
+      </c>
+      <c r="R88" t="n">
+        <v>60</v>
+      </c>
+      <c r="S88" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T88" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U88" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V88" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W88" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="n">
+        <v>45</v>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A10</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>ACEROMEX-64-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E89" t="n">
+        <v>4</v>
+      </c>
+      <c r="F89" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J89" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K89" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L89" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M89" t="n">
+        <v>48</v>
+      </c>
+      <c r="N89" t="n">
+        <v>120</v>
+      </c>
+      <c r="O89" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P89" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q89" t="n">
+        <v>0</v>
+      </c>
+      <c r="R89" t="n">
+        <v>60</v>
+      </c>
+      <c r="S89" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T89" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U89" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V89" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W89" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="n">
+        <v>45</v>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A11</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>ACEROMEX-63-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E90" t="n">
+        <v>1</v>
+      </c>
+      <c r="F90" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J90" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K90" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L90" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M90" t="n">
+        <v>48</v>
+      </c>
+      <c r="N90" t="n">
+        <v>120</v>
+      </c>
+      <c r="O90" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P90" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q90" t="n">
+        <v>0</v>
+      </c>
+      <c r="R90" t="n">
+        <v>60</v>
+      </c>
+      <c r="S90" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T90" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U90" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V90" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W90" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="n">
+        <v>45</v>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A11</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>ACEROMEX-63-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E91" t="n">
+        <v>2</v>
+      </c>
+      <c r="F91" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J91" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K91" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L91" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M91" t="n">
+        <v>48</v>
+      </c>
+      <c r="N91" t="n">
+        <v>120</v>
+      </c>
+      <c r="O91" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P91" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q91" t="n">
+        <v>0</v>
+      </c>
+      <c r="R91" t="n">
+        <v>60</v>
+      </c>
+      <c r="S91" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T91" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U91" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V91" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W91" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="n">
+        <v>45</v>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A11</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr">
+        <is>
+          <t>ACEROMEX-63-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E92" t="n">
+        <v>3</v>
+      </c>
+      <c r="F92" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J92" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K92" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L92" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M92" t="n">
+        <v>48</v>
+      </c>
+      <c r="N92" t="n">
+        <v>120</v>
+      </c>
+      <c r="O92" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P92" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q92" t="n">
+        <v>0</v>
+      </c>
+      <c r="R92" t="n">
+        <v>60</v>
+      </c>
+      <c r="S92" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T92" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U92" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V92" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W92" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="n">
+        <v>45</v>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A11</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr">
+        <is>
+          <t>ACEROMEX-63-2B485513GN</t>
+        </is>
+      </c>
+      <c r="E93" t="n">
+        <v>4</v>
+      </c>
+      <c r="F93" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J93" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L93" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M93" t="n">
+        <v>48</v>
+      </c>
+      <c r="N93" t="n">
+        <v>120</v>
+      </c>
+      <c r="O93" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P93" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>0</v>
+      </c>
+      <c r="R93" t="n">
+        <v>60</v>
+      </c>
+      <c r="S93" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T93" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U93" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V93" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W93" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="n">
+        <v>11</v>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A12</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr">
+        <is>
+          <t>ACEROMEX-60-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E94" t="n">
+        <v>1</v>
+      </c>
+      <c r="F94" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J94" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K94" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L94" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M94" t="n">
+        <v>48</v>
+      </c>
+      <c r="N94" t="n">
+        <v>120</v>
+      </c>
+      <c r="O94" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P94" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q94" t="n">
+        <v>0</v>
+      </c>
+      <c r="R94" t="n">
+        <v>60</v>
+      </c>
+      <c r="S94" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T94" t="inlineStr">
+        <is>
+          <t>Rayas/Manchas, Marcas de Rodillos</t>
+        </is>
+      </c>
+      <c r="U94" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V94" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="W94" t="inlineStr">
+        <is>
+          <t>Material con daños en el acabado (oxido)</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="n">
+        <v>11</v>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A12</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D95" t="inlineStr">
+        <is>
+          <t>ACEROMEX-60-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E95" t="n">
+        <v>2</v>
+      </c>
+      <c r="F95" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G95" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J95" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K95" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L95" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M95" t="n">
+        <v>48</v>
+      </c>
+      <c r="N95" t="n">
+        <v>120</v>
+      </c>
+      <c r="O95" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P95" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q95" t="n">
+        <v>0</v>
+      </c>
+      <c r="R95" t="n">
+        <v>60</v>
+      </c>
+      <c r="S95" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T95" t="inlineStr">
+        <is>
+          <t>Rayas/Manchas, Marcas de Rodillos</t>
+        </is>
+      </c>
+      <c r="U95" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V95" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="W95" t="inlineStr">
+        <is>
+          <t>Material con daños en el acabado (oxido)</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="n">
+        <v>11</v>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A12</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D96" t="inlineStr">
+        <is>
+          <t>ACEROMEX-60-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E96" t="n">
+        <v>3</v>
+      </c>
+      <c r="F96" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G96" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J96" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K96" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L96" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M96" t="n">
+        <v>48</v>
+      </c>
+      <c r="N96" t="n">
+        <v>120</v>
+      </c>
+      <c r="O96" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P96" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q96" t="n">
+        <v>0</v>
+      </c>
+      <c r="R96" t="n">
+        <v>60</v>
+      </c>
+      <c r="S96" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T96" t="inlineStr">
+        <is>
+          <t>Rayas/Manchas, Marcas de Rodillos</t>
+        </is>
+      </c>
+      <c r="U96" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V96" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="W96" t="inlineStr">
+        <is>
+          <t>Material con daños en el acabado (oxido)</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="n">
+        <v>11</v>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>INC-2026-0002-A12</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>INC-2026-0002</t>
+        </is>
+      </c>
+      <c r="D97" t="inlineStr">
+        <is>
+          <t>ACEROMEX-60-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E97" t="n">
+        <v>4</v>
+      </c>
+      <c r="F97" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G97" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J97" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K97" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L97" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M97" t="n">
+        <v>48</v>
+      </c>
+      <c r="N97" t="n">
+        <v>120</v>
+      </c>
+      <c r="O97" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P97" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q97" t="n">
+        <v>0</v>
+      </c>
+      <c r="R97" t="n">
+        <v>60</v>
+      </c>
+      <c r="S97" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T97" t="inlineStr">
+        <is>
+          <t>Rayas/Manchas, Marcas de Rodillos</t>
+        </is>
+      </c>
+      <c r="U97" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V97" t="inlineStr">
+        <is>
+          <t>Rechazado</t>
+        </is>
+      </c>
+      <c r="W97" t="inlineStr">
         <is>
           <t>Material con daños en el acabado (oxido)</t>
         </is>

</xml_diff>

<commit_message>
Auto-registro SGC: Folio INC-2026-0003
</commit_message>
<xml_diff>
--- a/BD_Atados_Incoming.xlsx
+++ b/BD_Atados_Incoming.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W97"/>
+  <dimension ref="A1:W117"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -9653,6 +9653,1906 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="n">
+        <v>45</v>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A01</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D98" t="inlineStr">
+        <is>
+          <t>ACEROMEX-55-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E98" t="n">
+        <v>1</v>
+      </c>
+      <c r="F98" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G98" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H98" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J98" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K98" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L98" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M98" t="n">
+        <v>48</v>
+      </c>
+      <c r="N98" t="n">
+        <v>120</v>
+      </c>
+      <c r="O98" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P98" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q98" t="n">
+        <v>0</v>
+      </c>
+      <c r="R98" t="n">
+        <v>60</v>
+      </c>
+      <c r="S98" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T98" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U98" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V98" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W98" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="n">
+        <v>45</v>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A01</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D99" t="inlineStr">
+        <is>
+          <t>ACEROMEX-55-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E99" t="n">
+        <v>2</v>
+      </c>
+      <c r="F99" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G99" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H99" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J99" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K99" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L99" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M99" t="n">
+        <v>48</v>
+      </c>
+      <c r="N99" t="n">
+        <v>120</v>
+      </c>
+      <c r="O99" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P99" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q99" t="n">
+        <v>0</v>
+      </c>
+      <c r="R99" t="n">
+        <v>60</v>
+      </c>
+      <c r="S99" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T99" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U99" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V99" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W99" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="n">
+        <v>45</v>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A01</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D100" t="inlineStr">
+        <is>
+          <t>ACEROMEX-55-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E100" t="n">
+        <v>3</v>
+      </c>
+      <c r="F100" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G100" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H100" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J100" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="K100" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="L100" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="M100" t="n">
+        <v>48</v>
+      </c>
+      <c r="N100" t="n">
+        <v>120</v>
+      </c>
+      <c r="O100" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P100" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q100" t="n">
+        <v>0</v>
+      </c>
+      <c r="R100" t="n">
+        <v>60</v>
+      </c>
+      <c r="S100" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T100" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U100" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V100" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W100" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="n">
+        <v>45</v>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A01</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D101" t="inlineStr">
+        <is>
+          <t>ACEROMEX-55-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E101" t="n">
+        <v>4</v>
+      </c>
+      <c r="F101" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G101" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H101" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J101" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K101" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L101" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M101" t="n">
+        <v>48</v>
+      </c>
+      <c r="N101" t="n">
+        <v>120</v>
+      </c>
+      <c r="O101" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P101" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q101" t="n">
+        <v>0</v>
+      </c>
+      <c r="R101" t="n">
+        <v>60</v>
+      </c>
+      <c r="S101" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T101" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U101" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V101" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W101" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="n">
+        <v>45</v>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A02</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D102" t="inlineStr">
+        <is>
+          <t>ACEROMEX-56-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E102" t="n">
+        <v>1</v>
+      </c>
+      <c r="F102" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G102" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H102" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J102" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="K102" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L102" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="M102" t="n">
+        <v>48</v>
+      </c>
+      <c r="N102" t="n">
+        <v>120</v>
+      </c>
+      <c r="O102" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P102" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q102" t="n">
+        <v>0</v>
+      </c>
+      <c r="R102" t="n">
+        <v>60</v>
+      </c>
+      <c r="S102" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T102" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U102" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V102" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W102" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="n">
+        <v>45</v>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A02</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D103" t="inlineStr">
+        <is>
+          <t>ACEROMEX-56-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E103" t="n">
+        <v>2</v>
+      </c>
+      <c r="F103" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G103" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H103" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J103" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K103" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L103" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M103" t="n">
+        <v>48</v>
+      </c>
+      <c r="N103" t="n">
+        <v>120</v>
+      </c>
+      <c r="O103" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P103" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q103" t="n">
+        <v>0</v>
+      </c>
+      <c r="R103" t="n">
+        <v>60</v>
+      </c>
+      <c r="S103" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T103" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U103" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V103" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W103" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="n">
+        <v>45</v>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A02</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D104" t="inlineStr">
+        <is>
+          <t>ACEROMEX-56-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E104" t="n">
+        <v>3</v>
+      </c>
+      <c r="F104" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G104" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H104" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J104" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K104" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L104" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M104" t="n">
+        <v>48</v>
+      </c>
+      <c r="N104" t="n">
+        <v>120</v>
+      </c>
+      <c r="O104" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P104" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q104" t="n">
+        <v>0</v>
+      </c>
+      <c r="R104" t="n">
+        <v>60</v>
+      </c>
+      <c r="S104" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T104" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U104" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V104" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W104" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="n">
+        <v>45</v>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A02</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D105" t="inlineStr">
+        <is>
+          <t>ACEROMEX-56-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E105" t="n">
+        <v>4</v>
+      </c>
+      <c r="F105" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G105" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H105" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J105" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K105" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L105" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M105" t="n">
+        <v>48</v>
+      </c>
+      <c r="N105" t="n">
+        <v>120</v>
+      </c>
+      <c r="O105" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P105" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q105" t="n">
+        <v>0</v>
+      </c>
+      <c r="R105" t="n">
+        <v>60</v>
+      </c>
+      <c r="S105" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T105" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U105" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V105" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W105" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="n">
+        <v>45</v>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A03</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D106" t="inlineStr">
+        <is>
+          <t>ACEROMEX-61-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E106" t="n">
+        <v>1</v>
+      </c>
+      <c r="F106" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G106" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H106" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J106" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K106" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L106" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M106" t="n">
+        <v>48</v>
+      </c>
+      <c r="N106" t="n">
+        <v>120</v>
+      </c>
+      <c r="O106" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P106" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q106" t="n">
+        <v>0</v>
+      </c>
+      <c r="R106" t="n">
+        <v>60</v>
+      </c>
+      <c r="S106" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T106" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U106" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V106" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W106" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="n">
+        <v>45</v>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A03</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D107" t="inlineStr">
+        <is>
+          <t>ACEROMEX-61-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E107" t="n">
+        <v>2</v>
+      </c>
+      <c r="F107" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G107" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H107" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J107" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K107" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="L107" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="M107" t="n">
+        <v>48</v>
+      </c>
+      <c r="N107" t="n">
+        <v>120</v>
+      </c>
+      <c r="O107" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P107" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q107" t="n">
+        <v>0</v>
+      </c>
+      <c r="R107" t="n">
+        <v>60</v>
+      </c>
+      <c r="S107" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T107" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U107" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V107" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W107" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="n">
+        <v>45</v>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A03</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D108" t="inlineStr">
+        <is>
+          <t>ACEROMEX-61-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E108" t="n">
+        <v>3</v>
+      </c>
+      <c r="F108" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G108" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H108" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J108" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K108" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L108" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M108" t="n">
+        <v>48</v>
+      </c>
+      <c r="N108" t="n">
+        <v>120</v>
+      </c>
+      <c r="O108" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P108" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q108" t="n">
+        <v>0</v>
+      </c>
+      <c r="R108" t="n">
+        <v>60</v>
+      </c>
+      <c r="S108" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T108" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U108" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V108" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W108" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="n">
+        <v>45</v>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A03</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D109" t="inlineStr">
+        <is>
+          <t>ACEROMEX-61-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E109" t="n">
+        <v>4</v>
+      </c>
+      <c r="F109" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G109" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H109" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J109" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K109" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="L109" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="M109" t="n">
+        <v>48</v>
+      </c>
+      <c r="N109" t="n">
+        <v>120</v>
+      </c>
+      <c r="O109" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P109" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q109" t="n">
+        <v>0</v>
+      </c>
+      <c r="R109" t="n">
+        <v>60</v>
+      </c>
+      <c r="S109" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T109" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U109" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V109" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W109" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="n">
+        <v>45</v>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A04</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D110" t="inlineStr">
+        <is>
+          <t>ACEROMEX-62-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E110" t="n">
+        <v>1</v>
+      </c>
+      <c r="F110" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G110" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H110" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J110" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K110" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L110" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M110" t="n">
+        <v>48</v>
+      </c>
+      <c r="N110" t="n">
+        <v>120</v>
+      </c>
+      <c r="O110" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P110" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q110" t="n">
+        <v>0</v>
+      </c>
+      <c r="R110" t="n">
+        <v>60</v>
+      </c>
+      <c r="S110" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T110" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U110" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V110" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W110" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="n">
+        <v>45</v>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A04</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D111" t="inlineStr">
+        <is>
+          <t>ACEROMEX-62-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E111" t="n">
+        <v>2</v>
+      </c>
+      <c r="F111" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G111" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H111" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J111" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K111" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="L111" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="M111" t="n">
+        <v>48</v>
+      </c>
+      <c r="N111" t="n">
+        <v>120</v>
+      </c>
+      <c r="O111" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P111" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q111" t="n">
+        <v>0</v>
+      </c>
+      <c r="R111" t="n">
+        <v>60</v>
+      </c>
+      <c r="S111" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T111" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U111" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V111" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W111" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="n">
+        <v>45</v>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A04</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D112" t="inlineStr">
+        <is>
+          <t>ACEROMEX-62-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E112" t="n">
+        <v>3</v>
+      </c>
+      <c r="F112" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G112" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H112" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J112" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K112" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L112" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M112" t="n">
+        <v>48</v>
+      </c>
+      <c r="N112" t="n">
+        <v>120</v>
+      </c>
+      <c r="O112" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P112" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q112" t="n">
+        <v>0</v>
+      </c>
+      <c r="R112" t="n">
+        <v>60</v>
+      </c>
+      <c r="S112" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T112" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U112" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V112" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W112" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="n">
+        <v>45</v>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A04</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D113" t="inlineStr">
+        <is>
+          <t>ACEROMEX-62-2B472917GN</t>
+        </is>
+      </c>
+      <c r="E113" t="n">
+        <v>4</v>
+      </c>
+      <c r="F113" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G113" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H113" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J113" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K113" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="L113" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="M113" t="n">
+        <v>48</v>
+      </c>
+      <c r="N113" t="n">
+        <v>120</v>
+      </c>
+      <c r="O113" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P113" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q113" t="n">
+        <v>0</v>
+      </c>
+      <c r="R113" t="n">
+        <v>60</v>
+      </c>
+      <c r="S113" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T113" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U113" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V113" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W113" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="n">
+        <v>45</v>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A05</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D114" t="inlineStr">
+        <is>
+          <t>ACEROMEX-65-52B472917GN</t>
+        </is>
+      </c>
+      <c r="E114" t="n">
+        <v>1</v>
+      </c>
+      <c r="F114" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G114" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H114" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J114" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="K114" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="L114" t="n">
+        <v>0.06</v>
+      </c>
+      <c r="M114" t="n">
+        <v>48</v>
+      </c>
+      <c r="N114" t="n">
+        <v>120</v>
+      </c>
+      <c r="O114" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P114" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q114" t="n">
+        <v>0</v>
+      </c>
+      <c r="R114" t="n">
+        <v>60</v>
+      </c>
+      <c r="S114" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T114" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U114" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V114" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W114" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="n">
+        <v>45</v>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A05</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D115" t="inlineStr">
+        <is>
+          <t>ACEROMEX-65-52B472917GN</t>
+        </is>
+      </c>
+      <c r="E115" t="n">
+        <v>2</v>
+      </c>
+      <c r="F115" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G115" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H115" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J115" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K115" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L115" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M115" t="n">
+        <v>48</v>
+      </c>
+      <c r="N115" t="n">
+        <v>120</v>
+      </c>
+      <c r="O115" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P115" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q115" t="n">
+        <v>0</v>
+      </c>
+      <c r="R115" t="n">
+        <v>60</v>
+      </c>
+      <c r="S115" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T115" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U115" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V115" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W115" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="n">
+        <v>45</v>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A05</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D116" t="inlineStr">
+        <is>
+          <t>ACEROMEX-65-52B472917GN</t>
+        </is>
+      </c>
+      <c r="E116" t="n">
+        <v>3</v>
+      </c>
+      <c r="F116" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G116" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H116" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J116" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="K116" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="L116" t="n">
+        <v>0.058</v>
+      </c>
+      <c r="M116" t="n">
+        <v>48</v>
+      </c>
+      <c r="N116" t="n">
+        <v>120</v>
+      </c>
+      <c r="O116" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P116" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q116" t="n">
+        <v>0</v>
+      </c>
+      <c r="R116" t="n">
+        <v>60</v>
+      </c>
+      <c r="S116" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T116" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U116" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V116" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W116" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="n">
+        <v>45</v>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>INC-2026-0003-A05</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>INC-2026-0003</t>
+        </is>
+      </c>
+      <c r="D117" t="inlineStr">
+        <is>
+          <t>ACEROMEX-65-52B472917GN</t>
+        </is>
+      </c>
+      <c r="E117" t="n">
+        <v>4</v>
+      </c>
+      <c r="F117" t="inlineStr">
+        <is>
+          <t>SKU-DECP-16</t>
+        </is>
+      </c>
+      <c r="G117" t="inlineStr">
+        <is>
+          <t>SAE 1008 CS</t>
+        </is>
+      </c>
+      <c r="H117" t="inlineStr">
+        <is>
+          <t>COL-2603210220</t>
+        </is>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>LOT-23687</t>
+        </is>
+      </c>
+      <c r="J117" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="K117" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="L117" t="n">
+        <v>0.059</v>
+      </c>
+      <c r="M117" t="n">
+        <v>48</v>
+      </c>
+      <c r="N117" t="n">
+        <v>120</v>
+      </c>
+      <c r="O117" t="n">
+        <v>2029</v>
+      </c>
+      <c r="P117" t="n">
+        <v>4473.2</v>
+      </c>
+      <c r="Q117" t="n">
+        <v>0</v>
+      </c>
+      <c r="R117" t="n">
+        <v>60</v>
+      </c>
+      <c r="S117" t="inlineStr">
+        <is>
+          <t>Sí</t>
+        </is>
+      </c>
+      <c r="T117" t="inlineStr">
+        <is>
+          <t>Ninguno</t>
+        </is>
+      </c>
+      <c r="U117" t="inlineStr">
+        <is>
+          <t>Almacén Metales</t>
+        </is>
+      </c>
+      <c r="V117" t="inlineStr">
+        <is>
+          <t>Aceptado</t>
+        </is>
+      </c>
+      <c r="W117" t="inlineStr">
+        <is>
+          <t>Excelente estado superficial</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>